<commit_message>
Align volume breakout operation scoring
Squash merge PR #135 after successful branch Daily Full Pipeline run 27736763773 and Research Backtest Pipeline run 27737354600.
</commit_message>
<xml_diff>
--- a/output/latest/stock_theme_manual_fill_template_latest.xlsx
+++ b/output/latest/stock_theme_manual_fill_template_latest.xlsx
@@ -86454,12 +86454,12 @@
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>其他業</t>
         </is>
       </c>
       <c r="D358" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>其他業</t>
         </is>
       </c>
       <c r="E358" t="inlineStr">

</xml_diff>

<commit_message>
Fix volume breakout operation PDF states
</commit_message>
<xml_diff>
--- a/output/latest/stock_theme_manual_fill_template_latest.xlsx
+++ b/output/latest/stock_theme_manual_fill_template_latest.xlsx
@@ -22,13 +22,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -39,7 +42,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -47,12 +50,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -426,12 +438,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>欄位</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>填寫方式</t>
         </is>
@@ -513,57 +525,57 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>股票代號</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>股票名稱</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>上市櫃產業</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>基本族群</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>主流/非主流</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>熱門族群1</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>熱門族群2</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>熱門族群3</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>熱門族群4</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>熱門族群5</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>備註</t>
         </is>
@@ -18617,57 +18629,57 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>股票代號</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>股票名稱</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>上市櫃產業</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>基本族群</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>主流/非主流</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>熱門族群1</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>熱門族群2</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>熱門族群3</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>熱門族群4</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>熱門族群5</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>備註</t>
         </is>
@@ -37377,57 +37389,57 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>股票代號</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>股票名稱</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>上市櫃產業</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>基本族群</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>主流/非主流</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>熱門族群1</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>熱門族群2</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>熱門族群3</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>熱門族群4</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>熱門族群5</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>備註</t>
         </is>
@@ -55957,57 +55969,57 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>股票代號</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>股票名稱</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>上市櫃產業</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>基本族群</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>主流/非主流</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>熱門族群1</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>熱門族群2</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>熱門族群3</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>熱門族群4</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>熱門族群5</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>備註</t>
         </is>
@@ -73805,57 +73817,57 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>股票代號</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>股票名稱</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>上市櫃產業</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>基本族群</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>主流/非主流</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>熱門族群1</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>熱門族群2</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>熱門族群3</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>熱門族群4</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>熱門族群5</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>備註</t>
         </is>

</xml_diff>

<commit_message>
Fix official price history continuity gate
* Fix official price history continuity gate

* Update daily report artifacts and packets

* Publish daily report readme and ChatGPT entries

---------

Co-authored-by: Codex <codex@local>
Co-authored-by: github-actions <github-actions@github.com>
</commit_message>
<xml_diff>
--- a/output/latest/stock_theme_manual_fill_template_latest.xlsx
+++ b/output/latest/stock_theme_manual_fill_template_latest.xlsx
@@ -16339,12 +16339,12 @@
       </c>
       <c r="C443" t="inlineStr">
         <is>
-          <t>其他業</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="D443" t="inlineStr">
         <is>
-          <t>其他業</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="E443" t="inlineStr">
@@ -23699,12 +23699,12 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>其他業</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>其他業</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
@@ -32097,12 +32097,12 @@
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>其他業</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="D361" t="inlineStr">
         <is>
-          <t>其他業</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="E361" t="inlineStr">
@@ -42400,12 +42400,12 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>其他業</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>其他業</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
@@ -48805,12 +48805,12 @@
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>其他業</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>其他業</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="E309" t="inlineStr">
@@ -51958,12 +51958,12 @@
       </c>
       <c r="C394" t="inlineStr">
         <is>
-          <t>金融保險業</t>
+          <t>金融業</t>
         </is>
       </c>
       <c r="D394" t="inlineStr">
         <is>
-          <t>金融保險業</t>
+          <t>金融業</t>
         </is>
       </c>
       <c r="E394" t="inlineStr">
@@ -52386,12 +52386,12 @@
       </c>
       <c r="C406" t="inlineStr">
         <is>
-          <t>金融保險業</t>
+          <t>金融業</t>
         </is>
       </c>
       <c r="D406" t="inlineStr">
         <is>
-          <t>金融保險業</t>
+          <t>金融業</t>
         </is>
       </c>
       <c r="E406" t="inlineStr">
@@ -52423,12 +52423,12 @@
       </c>
       <c r="C407" t="inlineStr">
         <is>
-          <t>金融保險業</t>
+          <t>金融業</t>
         </is>
       </c>
       <c r="D407" t="inlineStr">
         <is>
-          <t>金融保險業</t>
+          <t>金融業</t>
         </is>
       </c>
       <c r="E407" t="inlineStr">
@@ -52608,12 +52608,12 @@
       </c>
       <c r="C412" t="inlineStr">
         <is>
-          <t>金融保險業</t>
+          <t>金融業</t>
         </is>
       </c>
       <c r="D412" t="inlineStr">
         <is>
-          <t>金融保險業</t>
+          <t>金融業</t>
         </is>
       </c>
       <c r="E412" t="inlineStr">
@@ -54943,12 +54943,12 @@
       </c>
       <c r="C475" t="inlineStr">
         <is>
-          <t>其他業</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="D475" t="inlineStr">
         <is>
-          <t>其他業</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="E475" t="inlineStr">
@@ -55609,12 +55609,12 @@
       </c>
       <c r="C493" t="inlineStr">
         <is>
-          <t>其他業</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="D493" t="inlineStr">
         <is>
-          <t>其他業</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="E493" t="inlineStr">
@@ -84926,12 +84926,12 @@
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>其他業</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>其他業</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
@@ -85243,12 +85243,12 @@
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>DR / 外國上市</t>
+          <t>存託憑證</t>
         </is>
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>DR / 外國上市</t>
+          <t>存託憑證</t>
         </is>
       </c>
       <c r="E323" t="inlineStr">
@@ -85261,11 +85261,7 @@
       <c r="H323" t="inlineStr"/>
       <c r="I323" t="inlineStr"/>
       <c r="J323" t="inlineStr"/>
-      <c r="K323" t="inlineStr">
-        <is>
-          <t>provisional_industry_mapping</t>
-        </is>
-      </c>
+      <c r="K323" t="inlineStr"/>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">

</xml_diff>

<commit_message>
Harden volume breakout lifecycle source gaps
Harden volume breakout operation lifecycle lineage handling. Audit source gaps instead of silently dropping missing price-history evidence, avoid duplicate-source overwrite in signal history, and add tests/validators for source-gap audit semantics. Verified research backtest pipeline and daily full pipeline on the PR branch.
</commit_message>
<xml_diff>
--- a/output/latest/stock_theme_manual_fill_template_latest.xlsx
+++ b/output/latest/stock_theme_manual_fill_template_latest.xlsx
@@ -16339,12 +16339,12 @@
       </c>
       <c r="C443" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>其他業</t>
         </is>
       </c>
       <c r="D443" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>其他業</t>
         </is>
       </c>
       <c r="E443" t="inlineStr">
@@ -32097,12 +32097,12 @@
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>其他業</t>
         </is>
       </c>
       <c r="D361" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>其他業</t>
         </is>
       </c>
       <c r="E361" t="inlineStr">
@@ -42400,12 +42400,12 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>其他業</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>其他業</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
@@ -48805,12 +48805,12 @@
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>其他業</t>
         </is>
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>其他業</t>
         </is>
       </c>
       <c r="E309" t="inlineStr">
@@ -51958,12 +51958,12 @@
       </c>
       <c r="C394" t="inlineStr">
         <is>
-          <t>金融業</t>
+          <t>金融保險業</t>
         </is>
       </c>
       <c r="D394" t="inlineStr">
         <is>
-          <t>金融業</t>
+          <t>金融保險業</t>
         </is>
       </c>
       <c r="E394" t="inlineStr">
@@ -52386,12 +52386,12 @@
       </c>
       <c r="C406" t="inlineStr">
         <is>
-          <t>金融業</t>
+          <t>金融保險業</t>
         </is>
       </c>
       <c r="D406" t="inlineStr">
         <is>
-          <t>金融業</t>
+          <t>金融保險業</t>
         </is>
       </c>
       <c r="E406" t="inlineStr">
@@ -52423,12 +52423,12 @@
       </c>
       <c r="C407" t="inlineStr">
         <is>
-          <t>金融業</t>
+          <t>金融保險業</t>
         </is>
       </c>
       <c r="D407" t="inlineStr">
         <is>
-          <t>金融業</t>
+          <t>金融保險業</t>
         </is>
       </c>
       <c r="E407" t="inlineStr">
@@ -52608,12 +52608,12 @@
       </c>
       <c r="C412" t="inlineStr">
         <is>
-          <t>金融業</t>
+          <t>金融保險業</t>
         </is>
       </c>
       <c r="D412" t="inlineStr">
         <is>
-          <t>金融業</t>
+          <t>金融保險業</t>
         </is>
       </c>
       <c r="E412" t="inlineStr">
@@ -54943,12 +54943,12 @@
       </c>
       <c r="C475" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>其他業</t>
         </is>
       </c>
       <c r="D475" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>其他業</t>
         </is>
       </c>
       <c r="E475" t="inlineStr">
@@ -55609,12 +55609,12 @@
       </c>
       <c r="C493" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>其他業</t>
         </is>
       </c>
       <c r="D493" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>其他業</t>
         </is>
       </c>
       <c r="E493" t="inlineStr">
@@ -84926,12 +84926,12 @@
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>其他業</t>
         </is>
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>其他業</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
@@ -85243,12 +85243,12 @@
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>存託憑證</t>
+          <t>DR / 外國上市</t>
         </is>
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>存託憑證</t>
+          <t>DR / 外國上市</t>
         </is>
       </c>
       <c r="E323" t="inlineStr">
@@ -85261,7 +85261,11 @@
       <c r="H323" t="inlineStr"/>
       <c r="I323" t="inlineStr"/>
       <c r="J323" t="inlineStr"/>
-      <c r="K323" t="inlineStr"/>
+      <c r="K323" t="inlineStr">
+        <is>
+          <t>provisional_industry_mapping</t>
+        </is>
+      </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
@@ -86487,12 +86491,12 @@
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>其他業</t>
         </is>
       </c>
       <c r="D359" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>其他業</t>
         </is>
       </c>
       <c r="E359" t="inlineStr">
@@ -86520,12 +86524,12 @@
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>其他業</t>
         </is>
       </c>
       <c r="D360" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>其他業</t>
         </is>
       </c>
       <c r="E360" t="inlineStr">

</xml_diff>

<commit_message>
Harden daily external source gate ordering
Move full advanced integrity external-source validation until after daily catalyst source refresh, keep preflight boundary validation on static advanced contracts, refresh calendar source artifacts, and rebuild volume breakout formal/daily artifacts plus snapshots. Verified full local tests, Research Backtest Pipeline, and Daily Full Pipeline on the PR branch.
</commit_message>
<xml_diff>
--- a/output/latest/stock_theme_manual_fill_template_latest.xlsx
+++ b/output/latest/stock_theme_manual_fill_template_latest.xlsx
@@ -16339,12 +16339,12 @@
       </c>
       <c r="C443" t="inlineStr">
         <is>
-          <t>其他業</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="D443" t="inlineStr">
         <is>
-          <t>其他業</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="E443" t="inlineStr">
@@ -32097,12 +32097,12 @@
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>其他業</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="D361" t="inlineStr">
         <is>
-          <t>其他業</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="E361" t="inlineStr">
@@ -42400,12 +42400,12 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>其他業</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>其他業</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
@@ -48805,12 +48805,12 @@
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>其他業</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>其他業</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="E309" t="inlineStr">
@@ -51958,12 +51958,12 @@
       </c>
       <c r="C394" t="inlineStr">
         <is>
-          <t>金融保險業</t>
+          <t>金融業</t>
         </is>
       </c>
       <c r="D394" t="inlineStr">
         <is>
-          <t>金融保險業</t>
+          <t>金融業</t>
         </is>
       </c>
       <c r="E394" t="inlineStr">
@@ -52386,12 +52386,12 @@
       </c>
       <c r="C406" t="inlineStr">
         <is>
-          <t>金融保險業</t>
+          <t>金融業</t>
         </is>
       </c>
       <c r="D406" t="inlineStr">
         <is>
-          <t>金融保險業</t>
+          <t>金融業</t>
         </is>
       </c>
       <c r="E406" t="inlineStr">
@@ -52423,12 +52423,12 @@
       </c>
       <c r="C407" t="inlineStr">
         <is>
-          <t>金融保險業</t>
+          <t>金融業</t>
         </is>
       </c>
       <c r="D407" t="inlineStr">
         <is>
-          <t>金融保險業</t>
+          <t>金融業</t>
         </is>
       </c>
       <c r="E407" t="inlineStr">
@@ -52608,12 +52608,12 @@
       </c>
       <c r="C412" t="inlineStr">
         <is>
-          <t>金融保險業</t>
+          <t>金融業</t>
         </is>
       </c>
       <c r="D412" t="inlineStr">
         <is>
-          <t>金融保險業</t>
+          <t>金融業</t>
         </is>
       </c>
       <c r="E412" t="inlineStr">
@@ -54943,12 +54943,12 @@
       </c>
       <c r="C475" t="inlineStr">
         <is>
-          <t>其他業</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="D475" t="inlineStr">
         <is>
-          <t>其他業</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="E475" t="inlineStr">
@@ -55609,12 +55609,12 @@
       </c>
       <c r="C493" t="inlineStr">
         <is>
-          <t>其他業</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="D493" t="inlineStr">
         <is>
-          <t>其他業</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="E493" t="inlineStr">
@@ -84926,12 +84926,12 @@
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>其他業</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>其他業</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
@@ -85243,12 +85243,12 @@
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>DR / 外國上市</t>
+          <t>存託憑證</t>
         </is>
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>DR / 外國上市</t>
+          <t>存託憑證</t>
         </is>
       </c>
       <c r="E323" t="inlineStr">
@@ -85261,11 +85261,7 @@
       <c r="H323" t="inlineStr"/>
       <c r="I323" t="inlineStr"/>
       <c r="J323" t="inlineStr"/>
-      <c r="K323" t="inlineStr">
-        <is>
-          <t>provisional_industry_mapping</t>
-        </is>
-      </c>
+      <c r="K323" t="inlineStr"/>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
@@ -86491,12 +86487,12 @@
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>其他業</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="D359" t="inlineStr">
         <is>
-          <t>其他業</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="E359" t="inlineStr">
@@ -86524,12 +86520,12 @@
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>其他業</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="D360" t="inlineStr">
         <is>
-          <t>其他業</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="E360" t="inlineStr">

</xml_diff>